<commit_message>
Added auto client folder creation
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
   <si>
     <t>Client Name</t>
   </si>
@@ -46,16 +46,25 @@
     <t>Ramesh</t>
   </si>
   <si>
+    <t>Rahul</t>
+  </si>
+  <si>
     <t>bhrpl6522e</t>
   </si>
   <si>
     <t>bhrpl6522d</t>
   </si>
   <si>
+    <t>jdnkn3737r</t>
+  </si>
+  <si>
     <t>36DCRPS5473P1ZC</t>
   </si>
   <si>
     <t>36DCRPS5473P1Ze</t>
+  </si>
+  <si>
+    <t>36kshdh2737nd24</t>
   </si>
   <si>
     <t>2026-27</t>
@@ -396,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -430,25 +439,25 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -456,25 +465,51 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
         <v>13</v>
       </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="C4" t="s">
         <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added document checklist generation
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="23">
   <si>
     <t>Client Name</t>
   </si>
@@ -49,6 +49,9 @@
     <t>Rahul</t>
   </si>
   <si>
+    <t>Raju</t>
+  </si>
+  <si>
     <t>bhrpl6522e</t>
   </si>
   <si>
@@ -58,6 +61,9 @@
     <t>jdnkn3737r</t>
   </si>
   <si>
+    <t>hshsh2727y</t>
+  </si>
+  <si>
     <t>36DCRPS5473P1ZC</t>
   </si>
   <si>
@@ -65,6 +71,9 @@
   </si>
   <si>
     <t>36kshdh2737nd24</t>
+  </si>
+  <si>
+    <t>sdvbksdjvskjvn</t>
   </si>
   <si>
     <t>2026-27</t>
@@ -405,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -439,25 +448,25 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -465,25 +474,25 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -491,25 +500,51 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
         <v>19</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added checklist completion tracking
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="27">
   <si>
     <t>Client Name</t>
   </si>
@@ -40,6 +40,9 @@
     <t>Assigned Staff</t>
   </si>
   <si>
+    <t>Checklist Completion %</t>
+  </si>
+  <si>
     <t>Abhishek</t>
   </si>
   <si>
@@ -52,6 +55,9 @@
     <t>Raju</t>
   </si>
   <si>
+    <t>lokesh</t>
+  </si>
+  <si>
     <t>bhrpl6522e</t>
   </si>
   <si>
@@ -64,6 +70,9 @@
     <t>hshsh2727y</t>
   </si>
   <si>
+    <t>hshsh2727h</t>
+  </si>
+  <si>
     <t>36DCRPS5473P1ZC</t>
   </si>
   <si>
@@ -74,6 +83,9 @@
   </si>
   <si>
     <t>sdvbksdjvskjvn</t>
+  </si>
+  <si>
+    <t>bchdvbsdvbk</t>
   </si>
   <si>
     <t>2026-27</t>
@@ -414,10 +426,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -442,109 +454,141 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
         <v>22</v>
       </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="3" spans="1:8">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
         <v>13</v>
       </c>
-      <c r="C3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B6" t="s">
         <v>18</v>
       </c>
-      <c r="D4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H5" t="s">
-        <v>22</v>
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added working papers tracker generation
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="33">
   <si>
     <t>Client Name</t>
   </si>
@@ -61,6 +61,9 @@
     <t>lokesh</t>
   </si>
   <si>
+    <t>Poojamani</t>
+  </si>
+  <si>
     <t>bhrpl6522e</t>
   </si>
   <si>
@@ -76,6 +79,9 @@
     <t>hshsh2727h</t>
   </si>
   <si>
+    <t>hshsh5252f</t>
+  </si>
+  <si>
     <t>36DCRPS5473P1ZC</t>
   </si>
   <si>
@@ -89,6 +95,9 @@
   </si>
   <si>
     <t>bchdvbsdvbk</t>
+  </si>
+  <si>
+    <t>hbdbvdhvbksdvk</t>
   </si>
   <si>
     <t>2026-27</t>
@@ -435,7 +444,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -475,28 +484,28 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="I2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -507,28 +516,28 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="I3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -539,28 +548,28 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="I4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -571,28 +580,28 @@
         <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="I5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="J5">
         <v>100</v>
@@ -603,30 +612,62 @@
         <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G6" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" t="s">
+        <v>31</v>
+      </c>
+      <c r="I6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
         <v>28</v>
       </c>
-      <c r="H6" t="s">
-        <v>28</v>
-      </c>
-      <c r="I6" t="s">
-        <v>29</v>
-      </c>
-      <c r="J6">
+      <c r="E7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H7" t="s">
+        <v>31</v>
+      </c>
+      <c r="I7" t="s">
+        <v>14</v>
+      </c>
+      <c r="J7">
         <v>0</v>
       </c>
     </row>

</xml_diff>